<commit_message>
chore: atualizar template de relatório de inadimplência
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planilhas/relatorio_inadimplencia_modelo.xlsx
+++ b/planilhas/relatorio_inadimplencia_modelo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karol/Documents/Dashboard-Ativuz/planilhas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66176049-6713-8C4D-9DEF-F30CC05A77F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28D8F955-52CB-7F4F-8375-B61105994BC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="40">
   <si>
     <t>RELATÓRIO DE INADIMPLÊNCIA</t>
   </si>
@@ -396,7 +396,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="34">
+  <borders count="37">
     <border>
       <left/>
       <right/>
@@ -803,12 +803,49 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFBDBDBD"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="117">
+  <cellXfs count="122">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -845,12 +882,6 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -897,7 +928,6 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
@@ -953,6 +983,126 @@
     <xf numFmtId="44" fontId="9" fillId="11" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -998,126 +1148,18 @@
     <xf numFmtId="44" fontId="7" fillId="9" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="35" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="36" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
@@ -1421,7 +1463,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J73"/>
+  <dimension ref="A1:J81"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="40.6640625" customWidth="1"/>
@@ -1435,82 +1477,82 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="8" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="47"/>
+      <c r="A1" s="44"/>
     </row>
     <row r="2" spans="1:9" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="47"/>
-      <c r="B2" s="83" t="s">
+      <c r="A2" s="44"/>
+      <c r="B2" s="85" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="84"/>
-      <c r="D2" s="84"/>
-      <c r="E2" s="84"/>
-      <c r="F2" s="84"/>
-      <c r="G2" s="84"/>
-      <c r="H2" s="84"/>
-      <c r="I2" s="84"/>
+      <c r="C2" s="86"/>
+      <c r="D2" s="86"/>
+      <c r="E2" s="86"/>
+      <c r="F2" s="86"/>
+      <c r="G2" s="86"/>
+      <c r="H2" s="86"/>
+      <c r="I2" s="86"/>
     </row>
     <row r="3" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="47"/>
-      <c r="B3" s="85" t="s">
+      <c r="A3" s="44"/>
+      <c r="B3" s="87" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="86"/>
-      <c r="D3" s="86"/>
-      <c r="E3" s="86"/>
-      <c r="F3" s="86"/>
-      <c r="G3" s="86"/>
-      <c r="H3" s="86"/>
-      <c r="I3" s="86"/>
+      <c r="C3" s="88"/>
+      <c r="D3" s="88"/>
+      <c r="E3" s="88"/>
+      <c r="F3" s="88"/>
+      <c r="G3" s="88"/>
+      <c r="H3" s="88"/>
+      <c r="I3" s="88"/>
     </row>
     <row r="4" spans="1:9" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="47"/>
-      <c r="B4" s="27" t="s">
+      <c r="A4" s="44"/>
+      <c r="B4" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="65" t="s">
+      <c r="C4" s="102" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="65"/>
-      <c r="E4" s="87" t="s">
+      <c r="D4" s="102"/>
+      <c r="E4" s="89" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="88"/>
-      <c r="G4" s="89"/>
-      <c r="H4" s="67" t="s">
+      <c r="F4" s="90"/>
+      <c r="G4" s="91"/>
+      <c r="H4" s="104" t="s">
         <v>5</v>
       </c>
-      <c r="I4" s="68"/>
+      <c r="I4" s="105"/>
     </row>
     <row r="5" spans="1:9" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="47"/>
-      <c r="B5" s="28">
-        <f>COUNTA(C9:C70)</f>
+      <c r="A5" s="44"/>
+      <c r="B5" s="26">
+        <f>COUNTA(C9:C78)</f>
         <v>5</v>
       </c>
-      <c r="C5" s="66">
-        <f>SUM(E9:E70)</f>
+      <c r="C5" s="103">
+        <f>SUM(E9:E78)</f>
         <v>498</v>
       </c>
-      <c r="D5" s="66"/>
-      <c r="E5" s="90">
-        <f>SUM(H9:H70)</f>
+      <c r="D5" s="103"/>
+      <c r="E5" s="92">
+        <f>SUM(H9:H78)</f>
         <v>1031.3</v>
       </c>
-      <c r="F5" s="91"/>
-      <c r="G5" s="92"/>
-      <c r="H5" s="69">
-        <f>SUM(I9:I70)</f>
+      <c r="F5" s="93"/>
+      <c r="G5" s="94"/>
+      <c r="H5" s="106">
+        <f>SUM(I9:I78)</f>
         <v>3291.3</v>
       </c>
-      <c r="I5" s="70"/>
+      <c r="I5" s="107"/>
     </row>
     <row r="6" spans="1:9" ht="10" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="47"/>
+      <c r="A6" s="44"/>
     </row>
     <row r="7" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="47"/>
-      <c r="B7" s="48" t="s">
+      <c r="A7" s="44"/>
+      <c r="B7" s="45" t="s">
         <v>6</v>
       </c>
       <c r="C7" s="3" t="s">
@@ -1522,25 +1564,25 @@
       <c r="E7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="93" t="s">
+      <c r="F7" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="G7" s="94"/>
+      <c r="G7" s="96"/>
       <c r="H7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="I7" s="29" t="s">
+      <c r="I7" s="27" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="47"/>
-      <c r="F8" s="40"/>
-      <c r="G8" s="40"/>
+      <c r="A8" s="44"/>
+      <c r="F8" s="37"/>
+      <c r="G8" s="37"/>
     </row>
     <row r="9" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="47"/>
-      <c r="B9" s="45" t="s">
+      <c r="A9" s="44"/>
+      <c r="B9" s="42" t="s">
         <v>12</v>
       </c>
       <c r="C9" s="1" t="s">
@@ -1552,20 +1594,20 @@
       <c r="E9" s="1">
         <v>218</v>
       </c>
-      <c r="F9" s="71">
+      <c r="F9" s="108">
         <v>30</v>
       </c>
-      <c r="G9" s="72"/>
-      <c r="H9" s="55">
+      <c r="G9" s="109"/>
+      <c r="H9" s="52">
         <v>32.700000000000003</v>
       </c>
-      <c r="I9" s="56">
+      <c r="I9" s="53">
         <v>62.7</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="47"/>
-      <c r="B10" s="46" t="s">
+      <c r="A10" s="44"/>
+      <c r="B10" s="43" t="s">
         <v>15</v>
       </c>
       <c r="C10" s="1" t="s">
@@ -1574,23 +1616,23 @@
       <c r="D10" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="44">
+      <c r="E10" s="41">
         <v>45</v>
       </c>
-      <c r="F10" s="73">
+      <c r="F10" s="110">
         <v>180</v>
       </c>
-      <c r="G10" s="74"/>
-      <c r="H10" s="57">
+      <c r="G10" s="111"/>
+      <c r="H10" s="54">
         <v>40.5</v>
       </c>
-      <c r="I10" s="56">
+      <c r="I10" s="53">
         <v>220.5</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="47"/>
-      <c r="B11" s="45" t="s">
+      <c r="A11" s="44"/>
+      <c r="B11" s="42" t="s">
         <v>17</v>
       </c>
       <c r="C11" s="1" t="s">
@@ -1599,23 +1641,23 @@
       <c r="D11" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="43">
+      <c r="E11" s="40">
         <v>88</v>
       </c>
-      <c r="F11" s="75">
+      <c r="F11" s="112">
         <v>500</v>
       </c>
-      <c r="G11" s="76"/>
-      <c r="H11" s="57">
+      <c r="G11" s="113"/>
+      <c r="H11" s="54">
         <v>220</v>
       </c>
-      <c r="I11" s="56">
+      <c r="I11" s="53">
         <v>720</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="47"/>
-      <c r="B12" s="46" t="s">
+      <c r="A12" s="44"/>
+      <c r="B12" s="43" t="s">
         <v>20</v>
       </c>
       <c r="C12" s="1" t="s">
@@ -1624,23 +1666,23 @@
       <c r="D12" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="43">
+      <c r="E12" s="40">
         <v>113</v>
       </c>
-      <c r="F12" s="75">
+      <c r="F12" s="112">
         <v>1200</v>
       </c>
-      <c r="G12" s="76"/>
-      <c r="H12" s="57">
+      <c r="G12" s="113"/>
+      <c r="H12" s="54">
         <v>678.6</v>
       </c>
-      <c r="I12" s="56">
+      <c r="I12" s="53">
         <v>1878.6</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="47"/>
-      <c r="B13" s="45" t="s">
+      <c r="A13" s="44"/>
+      <c r="B13" s="42" t="s">
         <v>23</v>
       </c>
       <c r="C13" s="1" t="s">
@@ -1649,744 +1691,774 @@
       <c r="D13" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="44">
+      <c r="E13" s="41">
         <v>34</v>
       </c>
-      <c r="F13" s="73">
+      <c r="F13" s="110">
         <v>350</v>
       </c>
-      <c r="G13" s="74"/>
-      <c r="H13" s="57">
+      <c r="G13" s="111"/>
+      <c r="H13" s="54">
         <v>59.5</v>
       </c>
-      <c r="I13" s="56">
+      <c r="I13" s="53">
         <v>409.5</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="47"/>
-      <c r="B14" s="33"/>
+      <c r="A14" s="44"/>
+      <c r="B14" s="31"/>
       <c r="C14" s="10"/>
       <c r="D14" s="10"/>
-      <c r="E14" s="30"/>
-      <c r="F14" s="77"/>
-      <c r="G14" s="78"/>
-      <c r="H14" s="33"/>
-      <c r="I14" s="41"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="71"/>
+      <c r="G14" s="72"/>
+      <c r="H14" s="31"/>
+      <c r="I14" s="38"/>
     </row>
     <row r="15" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="47"/>
-      <c r="B15" s="32"/>
+      <c r="A15" s="44"/>
+      <c r="B15" s="30"/>
       <c r="C15" s="11"/>
       <c r="D15" s="11"/>
-      <c r="E15" s="31"/>
-      <c r="F15" s="79"/>
-      <c r="G15" s="80"/>
-      <c r="H15" s="32"/>
-      <c r="I15" s="42"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="61"/>
+      <c r="G15" s="62"/>
+      <c r="H15" s="30"/>
+      <c r="I15" s="39"/>
     </row>
     <row r="16" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="47"/>
-      <c r="B16" s="33"/>
+      <c r="A16" s="44"/>
+      <c r="B16" s="31"/>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
-      <c r="E16" s="30"/>
-      <c r="F16" s="81"/>
-      <c r="G16" s="82"/>
-      <c r="H16" s="33"/>
-      <c r="I16" s="41"/>
+      <c r="E16" s="28"/>
+      <c r="F16" s="59"/>
+      <c r="G16" s="60"/>
+      <c r="H16" s="31"/>
+      <c r="I16" s="38"/>
     </row>
     <row r="17" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="47"/>
-      <c r="B17" s="32"/>
+      <c r="A17" s="44"/>
+      <c r="B17" s="30"/>
       <c r="C17" s="11"/>
       <c r="D17" s="11"/>
-      <c r="E17" s="31"/>
-      <c r="F17" s="79"/>
-      <c r="G17" s="80"/>
-      <c r="H17" s="32"/>
-      <c r="I17" s="42"/>
+      <c r="E17" s="29"/>
+      <c r="F17" s="61"/>
+      <c r="G17" s="62"/>
+      <c r="H17" s="30"/>
+      <c r="I17" s="39"/>
     </row>
     <row r="18" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="47"/>
-      <c r="B18" s="33"/>
+      <c r="A18" s="44"/>
+      <c r="B18" s="31"/>
       <c r="C18" s="10"/>
       <c r="D18" s="10"/>
-      <c r="E18" s="30"/>
-      <c r="F18" s="81"/>
-      <c r="G18" s="82"/>
-      <c r="H18" s="33"/>
-      <c r="I18" s="41"/>
+      <c r="E18" s="28"/>
+      <c r="F18" s="59"/>
+      <c r="G18" s="60"/>
+      <c r="H18" s="31"/>
+      <c r="I18" s="38"/>
     </row>
     <row r="19" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="47"/>
-      <c r="B19" s="32"/>
+      <c r="A19" s="44"/>
+      <c r="B19" s="30"/>
       <c r="C19" s="11"/>
       <c r="D19" s="11"/>
       <c r="E19" s="11"/>
-      <c r="F19" s="95"/>
-      <c r="G19" s="96"/>
+      <c r="F19" s="83"/>
+      <c r="G19" s="84"/>
       <c r="H19" s="11"/>
-      <c r="I19" s="42"/>
+      <c r="I19" s="39"/>
     </row>
     <row r="20" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="47"/>
-      <c r="B20" s="33"/>
+      <c r="A20" s="44"/>
+      <c r="B20" s="31"/>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
-      <c r="E20" s="30"/>
-      <c r="F20" s="81"/>
-      <c r="G20" s="82"/>
-      <c r="H20" s="33"/>
-      <c r="I20" s="41"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="59"/>
+      <c r="G20" s="60"/>
+      <c r="H20" s="31"/>
+      <c r="I20" s="38"/>
     </row>
     <row r="21" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="47"/>
-      <c r="B21" s="32"/>
+      <c r="A21" s="44"/>
+      <c r="B21" s="30"/>
       <c r="C21" s="11"/>
       <c r="D21" s="11"/>
-      <c r="E21" s="31"/>
-      <c r="F21" s="79"/>
-      <c r="G21" s="80"/>
-      <c r="H21" s="32"/>
-      <c r="I21" s="42"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="61"/>
+      <c r="G21" s="62"/>
+      <c r="H21" s="30"/>
+      <c r="I21" s="39"/>
     </row>
     <row r="22" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="47"/>
-      <c r="B22" s="33"/>
+      <c r="A22" s="44"/>
+      <c r="B22" s="31"/>
       <c r="C22" s="10"/>
       <c r="D22" s="10"/>
-      <c r="E22" s="30"/>
-      <c r="F22" s="81"/>
-      <c r="G22" s="82"/>
-      <c r="H22" s="33"/>
-      <c r="I22" s="41"/>
+      <c r="E22" s="28"/>
+      <c r="F22" s="59"/>
+      <c r="G22" s="60"/>
+      <c r="H22" s="31"/>
+      <c r="I22" s="38"/>
     </row>
     <row r="23" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="47"/>
-      <c r="B23" s="32"/>
+      <c r="A23" s="44"/>
+      <c r="B23" s="30"/>
       <c r="C23" s="11"/>
       <c r="D23" s="11"/>
-      <c r="E23" s="31"/>
-      <c r="F23" s="79"/>
-      <c r="G23" s="80"/>
-      <c r="H23" s="32"/>
-      <c r="I23" s="42"/>
+      <c r="E23" s="29"/>
+      <c r="F23" s="61"/>
+      <c r="G23" s="62"/>
+      <c r="H23" s="30"/>
+      <c r="I23" s="39"/>
     </row>
     <row r="24" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="47"/>
-      <c r="B24" s="33"/>
+      <c r="A24" s="44"/>
+      <c r="B24" s="31"/>
       <c r="C24" s="10"/>
       <c r="D24" s="10"/>
-      <c r="E24" s="30"/>
-      <c r="F24" s="81"/>
-      <c r="G24" s="82"/>
-      <c r="H24" s="33"/>
-      <c r="I24" s="41"/>
+      <c r="E24" s="28"/>
+      <c r="F24" s="59"/>
+      <c r="G24" s="60"/>
+      <c r="H24" s="31"/>
+      <c r="I24" s="38"/>
     </row>
     <row r="25" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="47"/>
-      <c r="B25" s="32"/>
+      <c r="A25" s="44"/>
+      <c r="B25" s="30"/>
       <c r="C25" s="11"/>
       <c r="D25" s="11"/>
       <c r="E25" s="11"/>
-      <c r="F25" s="95"/>
-      <c r="G25" s="96"/>
+      <c r="F25" s="83"/>
+      <c r="G25" s="84"/>
       <c r="H25" s="11"/>
-      <c r="I25" s="42"/>
+      <c r="I25" s="39"/>
     </row>
     <row r="26" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="47"/>
-      <c r="B26" s="33"/>
+      <c r="A26" s="44"/>
+      <c r="B26" s="31"/>
       <c r="C26" s="10"/>
       <c r="D26" s="10"/>
-      <c r="E26" s="30"/>
-      <c r="F26" s="77"/>
-      <c r="G26" s="78"/>
-      <c r="H26" s="33"/>
-      <c r="I26" s="41"/>
+      <c r="E26" s="28"/>
+      <c r="F26" s="71"/>
+      <c r="G26" s="72"/>
+      <c r="H26" s="31"/>
+      <c r="I26" s="38"/>
     </row>
     <row r="27" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="47"/>
-      <c r="B27" s="32"/>
+      <c r="A27" s="44"/>
+      <c r="B27" s="30"/>
       <c r="C27" s="11"/>
       <c r="D27" s="11"/>
-      <c r="E27" s="31"/>
-      <c r="F27" s="79"/>
-      <c r="G27" s="80"/>
-      <c r="H27" s="32"/>
-      <c r="I27" s="42"/>
+      <c r="E27" s="29"/>
+      <c r="F27" s="61"/>
+      <c r="G27" s="62"/>
+      <c r="H27" s="30"/>
+      <c r="I27" s="39"/>
     </row>
     <row r="28" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="47"/>
-      <c r="B28" s="33"/>
+      <c r="A28" s="44"/>
+      <c r="B28" s="31"/>
       <c r="C28" s="10"/>
       <c r="D28" s="10"/>
       <c r="E28" s="10"/>
-      <c r="F28" s="97"/>
-      <c r="G28" s="98"/>
+      <c r="F28" s="77"/>
+      <c r="G28" s="78"/>
       <c r="H28" s="10"/>
-      <c r="I28" s="41"/>
+      <c r="I28" s="38"/>
     </row>
     <row r="29" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="47"/>
-      <c r="B29" s="32"/>
+      <c r="A29" s="44"/>
+      <c r="B29" s="30"/>
       <c r="C29" s="11"/>
       <c r="D29" s="11"/>
       <c r="E29" s="11"/>
-      <c r="F29" s="99"/>
-      <c r="G29" s="100"/>
+      <c r="F29" s="79"/>
+      <c r="G29" s="80"/>
       <c r="H29" s="11"/>
-      <c r="I29" s="42"/>
+      <c r="I29" s="39"/>
     </row>
     <row r="30" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="47"/>
-      <c r="B30" s="33"/>
+      <c r="A30" s="44"/>
+      <c r="B30" s="31"/>
       <c r="C30" s="10"/>
       <c r="D30" s="10"/>
       <c r="E30" s="10"/>
-      <c r="F30" s="101"/>
-      <c r="G30" s="102"/>
+      <c r="F30" s="81"/>
+      <c r="G30" s="82"/>
       <c r="H30" s="10"/>
-      <c r="I30" s="41"/>
+      <c r="I30" s="38"/>
     </row>
     <row r="31" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="47"/>
-      <c r="B31" s="32"/>
+      <c r="A31" s="44"/>
+      <c r="B31" s="30"/>
       <c r="C31" s="11"/>
       <c r="D31" s="11"/>
-      <c r="E31" s="31"/>
-      <c r="F31" s="79"/>
-      <c r="G31" s="80"/>
-      <c r="H31" s="32"/>
-      <c r="I31" s="42"/>
+      <c r="E31" s="29"/>
+      <c r="F31" s="61"/>
+      <c r="G31" s="62"/>
+      <c r="H31" s="30"/>
+      <c r="I31" s="39"/>
     </row>
     <row r="32" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="47"/>
-      <c r="B32" s="33"/>
+      <c r="A32" s="44"/>
+      <c r="B32" s="31"/>
       <c r="C32" s="10"/>
       <c r="D32" s="10"/>
-      <c r="E32" s="30"/>
-      <c r="F32" s="103"/>
-      <c r="G32" s="104"/>
-      <c r="H32" s="33"/>
-      <c r="I32" s="41"/>
+      <c r="E32" s="28"/>
+      <c r="F32" s="67"/>
+      <c r="G32" s="68"/>
+      <c r="H32" s="31"/>
+      <c r="I32" s="38"/>
     </row>
     <row r="33" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="47"/>
-      <c r="B33" s="32"/>
+      <c r="A33" s="44"/>
+      <c r="B33" s="30"/>
       <c r="C33" s="11"/>
       <c r="D33" s="11"/>
       <c r="E33" s="11"/>
-      <c r="F33" s="99"/>
-      <c r="G33" s="100"/>
+      <c r="F33" s="79"/>
+      <c r="G33" s="80"/>
       <c r="H33" s="11"/>
-      <c r="I33" s="42"/>
+      <c r="I33" s="39"/>
     </row>
     <row r="34" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="47"/>
-      <c r="B34" s="33"/>
+      <c r="A34" s="44"/>
+      <c r="B34" s="31"/>
       <c r="C34" s="10"/>
       <c r="D34" s="10"/>
       <c r="E34" s="10"/>
-      <c r="F34" s="97"/>
-      <c r="G34" s="98"/>
+      <c r="F34" s="77"/>
+      <c r="G34" s="78"/>
       <c r="H34" s="10"/>
-      <c r="I34" s="41"/>
+      <c r="I34" s="38"/>
     </row>
     <row r="35" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="47"/>
-      <c r="B35" s="32"/>
+      <c r="A35" s="44"/>
+      <c r="B35" s="30"/>
       <c r="C35" s="11"/>
       <c r="D35" s="11"/>
       <c r="E35" s="11"/>
-      <c r="F35" s="99"/>
-      <c r="G35" s="100"/>
+      <c r="F35" s="79"/>
+      <c r="G35" s="80"/>
       <c r="H35" s="11"/>
-      <c r="I35" s="42"/>
+      <c r="I35" s="39"/>
     </row>
     <row r="36" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="47"/>
-      <c r="B36" s="33"/>
+      <c r="A36" s="44"/>
+      <c r="B36" s="31"/>
       <c r="C36" s="10"/>
       <c r="D36" s="10"/>
       <c r="E36" s="10"/>
-      <c r="F36" s="101"/>
-      <c r="G36" s="102"/>
+      <c r="F36" s="81"/>
+      <c r="G36" s="82"/>
       <c r="H36" s="10"/>
-      <c r="I36" s="41"/>
+      <c r="I36" s="38"/>
     </row>
     <row r="37" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="47"/>
-      <c r="B37" s="32"/>
+      <c r="A37" s="44"/>
+      <c r="B37" s="30"/>
       <c r="C37" s="11"/>
       <c r="D37" s="11"/>
       <c r="E37" s="11"/>
-      <c r="F37" s="99"/>
-      <c r="G37" s="100"/>
+      <c r="F37" s="79"/>
+      <c r="G37" s="80"/>
       <c r="H37" s="11"/>
-      <c r="I37" s="42"/>
+      <c r="I37" s="39"/>
     </row>
     <row r="38" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="47"/>
-      <c r="B38" s="33"/>
+      <c r="A38" s="44"/>
+      <c r="B38" s="31"/>
       <c r="C38" s="10"/>
       <c r="D38" s="10"/>
-      <c r="E38" s="30"/>
-      <c r="F38" s="77"/>
-      <c r="G38" s="78"/>
-      <c r="H38" s="33"/>
-      <c r="I38" s="41"/>
+      <c r="E38" s="28"/>
+      <c r="F38" s="71"/>
+      <c r="G38" s="72"/>
+      <c r="H38" s="31"/>
+      <c r="I38" s="38"/>
     </row>
     <row r="39" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="47"/>
-      <c r="B39" s="32"/>
+      <c r="A39" s="44"/>
+      <c r="B39" s="30"/>
       <c r="C39" s="11"/>
       <c r="D39" s="11"/>
-      <c r="E39" s="31"/>
-      <c r="F39" s="79"/>
-      <c r="G39" s="80"/>
-      <c r="H39" s="32"/>
-      <c r="I39" s="42"/>
+      <c r="E39" s="29"/>
+      <c r="F39" s="61"/>
+      <c r="G39" s="62"/>
+      <c r="H39" s="30"/>
+      <c r="I39" s="39"/>
     </row>
     <row r="40" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="47"/>
-      <c r="B40" s="33"/>
+      <c r="A40" s="44"/>
+      <c r="B40" s="31"/>
       <c r="C40" s="10"/>
       <c r="D40" s="10"/>
-      <c r="E40" s="30"/>
-      <c r="F40" s="77"/>
-      <c r="G40" s="78"/>
-      <c r="H40" s="33"/>
-      <c r="I40" s="41"/>
+      <c r="E40" s="28"/>
+      <c r="F40" s="71"/>
+      <c r="G40" s="72"/>
+      <c r="H40" s="31"/>
+      <c r="I40" s="38"/>
     </row>
     <row r="41" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="47"/>
-      <c r="B41" s="32"/>
+      <c r="A41" s="44"/>
+      <c r="B41" s="30"/>
       <c r="C41" s="11"/>
       <c r="D41" s="11"/>
-      <c r="E41" s="31"/>
-      <c r="F41" s="79"/>
-      <c r="G41" s="80"/>
-      <c r="H41" s="32"/>
-      <c r="I41" s="42"/>
+      <c r="E41" s="29"/>
+      <c r="F41" s="61"/>
+      <c r="G41" s="62"/>
+      <c r="H41" s="30"/>
+      <c r="I41" s="39"/>
     </row>
     <row r="42" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="47"/>
-      <c r="B42" s="33"/>
+      <c r="A42" s="44"/>
+      <c r="B42" s="31"/>
       <c r="C42" s="10"/>
       <c r="D42" s="10"/>
-      <c r="E42" s="30"/>
-      <c r="F42" s="105"/>
-      <c r="G42" s="106"/>
-      <c r="H42" s="33"/>
-      <c r="I42" s="41"/>
+      <c r="E42" s="28"/>
+      <c r="F42" s="73"/>
+      <c r="G42" s="74"/>
+      <c r="H42" s="31"/>
+      <c r="I42" s="38"/>
     </row>
     <row r="43" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="47"/>
-      <c r="B43" s="32"/>
+      <c r="A43" s="44"/>
+      <c r="B43" s="30"/>
       <c r="C43" s="11"/>
       <c r="D43" s="11"/>
-      <c r="E43" s="31"/>
-      <c r="F43" s="107"/>
-      <c r="G43" s="108"/>
-      <c r="H43" s="32"/>
-      <c r="I43" s="42"/>
+      <c r="E43" s="29"/>
+      <c r="F43" s="75"/>
+      <c r="G43" s="76"/>
+      <c r="H43" s="30"/>
+      <c r="I43" s="39"/>
     </row>
     <row r="44" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="47"/>
-      <c r="B44" s="33"/>
+      <c r="A44" s="44"/>
+      <c r="B44" s="31"/>
       <c r="C44" s="10"/>
       <c r="D44" s="10"/>
-      <c r="E44" s="30"/>
-      <c r="F44" s="81"/>
-      <c r="G44" s="82"/>
-      <c r="H44" s="33"/>
-      <c r="I44" s="41"/>
+      <c r="E44" s="28"/>
+      <c r="F44" s="59"/>
+      <c r="G44" s="60"/>
+      <c r="H44" s="31"/>
+      <c r="I44" s="38"/>
     </row>
     <row r="45" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="47"/>
-      <c r="B45" s="32"/>
+      <c r="A45" s="44"/>
+      <c r="B45" s="30"/>
       <c r="C45" s="11"/>
       <c r="D45" s="11"/>
-      <c r="E45" s="31"/>
-      <c r="F45" s="109"/>
-      <c r="G45" s="110"/>
-      <c r="H45" s="32"/>
-      <c r="I45" s="42"/>
+      <c r="E45" s="29"/>
+      <c r="F45" s="65"/>
+      <c r="G45" s="66"/>
+      <c r="H45" s="30"/>
+      <c r="I45" s="39"/>
     </row>
     <row r="46" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="47"/>
-      <c r="B46" s="33"/>
+      <c r="A46" s="44"/>
+      <c r="B46" s="31"/>
       <c r="C46" s="10"/>
       <c r="D46" s="10"/>
-      <c r="E46" s="30"/>
-      <c r="F46" s="105"/>
-      <c r="G46" s="106"/>
-      <c r="H46" s="33"/>
-      <c r="I46" s="41"/>
+      <c r="E46" s="28"/>
+      <c r="F46" s="73"/>
+      <c r="G46" s="74"/>
+      <c r="H46" s="31"/>
+      <c r="I46" s="38"/>
     </row>
     <row r="47" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="47"/>
-      <c r="B47" s="32"/>
+      <c r="A47" s="44"/>
+      <c r="B47" s="30"/>
       <c r="C47" s="11"/>
       <c r="D47" s="11"/>
-      <c r="E47" s="31"/>
-      <c r="F47" s="107"/>
-      <c r="G47" s="108"/>
-      <c r="H47" s="32"/>
-      <c r="I47" s="42"/>
+      <c r="E47" s="29"/>
+      <c r="F47" s="75"/>
+      <c r="G47" s="76"/>
+      <c r="H47" s="30"/>
+      <c r="I47" s="39"/>
     </row>
     <row r="48" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="47"/>
-      <c r="B48" s="33"/>
+      <c r="A48" s="44"/>
+      <c r="B48" s="31"/>
       <c r="C48" s="10"/>
       <c r="D48" s="10"/>
-      <c r="E48" s="30"/>
-      <c r="F48" s="81"/>
-      <c r="G48" s="82"/>
-      <c r="H48" s="33"/>
-      <c r="I48" s="41"/>
+      <c r="E48" s="28"/>
+      <c r="F48" s="59"/>
+      <c r="G48" s="60"/>
+      <c r="H48" s="31"/>
+      <c r="I48" s="38"/>
     </row>
     <row r="49" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="47"/>
-      <c r="B49" s="32"/>
+      <c r="A49" s="44"/>
+      <c r="B49" s="30"/>
       <c r="C49" s="11"/>
       <c r="D49" s="11"/>
-      <c r="E49" s="31"/>
-      <c r="F49" s="109"/>
-      <c r="G49" s="110"/>
-      <c r="H49" s="32"/>
-      <c r="I49" s="42"/>
+      <c r="E49" s="29"/>
+      <c r="F49" s="65"/>
+      <c r="G49" s="66"/>
+      <c r="H49" s="30"/>
+      <c r="I49" s="39"/>
     </row>
     <row r="50" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="47"/>
-      <c r="B50" s="33"/>
+      <c r="A50" s="44"/>
+      <c r="B50" s="31"/>
       <c r="C50" s="10"/>
       <c r="D50" s="10"/>
-      <c r="E50" s="30"/>
-      <c r="F50" s="103"/>
-      <c r="G50" s="104"/>
-      <c r="H50" s="33"/>
-      <c r="I50" s="41"/>
+      <c r="E50" s="28"/>
+      <c r="F50" s="67"/>
+      <c r="G50" s="68"/>
+      <c r="H50" s="31"/>
+      <c r="I50" s="38"/>
     </row>
     <row r="51" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="47"/>
-      <c r="B51" s="32"/>
+      <c r="A51" s="44"/>
+      <c r="B51" s="30"/>
       <c r="C51" s="11"/>
       <c r="D51" s="11"/>
       <c r="E51" s="11"/>
-      <c r="F51" s="111"/>
-      <c r="G51" s="112"/>
+      <c r="F51" s="69"/>
+      <c r="G51" s="70"/>
       <c r="H51" s="11"/>
-      <c r="I51" s="42"/>
+      <c r="I51" s="39"/>
     </row>
     <row r="52" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="47"/>
-      <c r="B52" s="33"/>
+      <c r="A52" s="44"/>
+      <c r="B52" s="31"/>
       <c r="C52" s="10"/>
       <c r="D52" s="10"/>
-      <c r="E52" s="30"/>
-      <c r="F52" s="103"/>
-      <c r="G52" s="104"/>
-      <c r="H52" s="33"/>
-      <c r="I52" s="41"/>
+      <c r="E52" s="28"/>
+      <c r="F52" s="67"/>
+      <c r="G52" s="68"/>
+      <c r="H52" s="31"/>
+      <c r="I52" s="38"/>
     </row>
     <row r="53" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="47"/>
-      <c r="B53" s="32"/>
+      <c r="A53" s="44"/>
+      <c r="B53" s="30"/>
       <c r="C53" s="11"/>
       <c r="D53" s="11"/>
       <c r="E53" s="11"/>
-      <c r="F53" s="111"/>
-      <c r="G53" s="112"/>
+      <c r="F53" s="69"/>
+      <c r="G53" s="70"/>
       <c r="H53" s="11"/>
-      <c r="I53" s="42"/>
+      <c r="I53" s="39"/>
     </row>
     <row r="54" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="47"/>
-      <c r="B54" s="33"/>
+      <c r="A54" s="44"/>
+      <c r="B54" s="31"/>
       <c r="C54" s="10"/>
       <c r="D54" s="10"/>
-      <c r="E54" s="30"/>
-      <c r="F54" s="103"/>
-      <c r="G54" s="104"/>
-      <c r="H54" s="33"/>
-      <c r="I54" s="41"/>
+      <c r="E54" s="28"/>
+      <c r="F54" s="67"/>
+      <c r="G54" s="68"/>
+      <c r="H54" s="31"/>
+      <c r="I54" s="38"/>
     </row>
     <row r="55" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="47"/>
-      <c r="B55" s="32"/>
+      <c r="A55" s="44"/>
+      <c r="B55" s="30"/>
       <c r="C55" s="11"/>
       <c r="D55" s="11"/>
       <c r="E55" s="11"/>
-      <c r="F55" s="111"/>
-      <c r="G55" s="112"/>
+      <c r="F55" s="69"/>
+      <c r="G55" s="70"/>
       <c r="H55" s="11"/>
-      <c r="I55" s="42"/>
+      <c r="I55" s="39"/>
     </row>
     <row r="56" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="47"/>
-      <c r="B56" s="33"/>
+      <c r="A56" s="44"/>
+      <c r="B56" s="31"/>
       <c r="C56" s="10"/>
       <c r="D56" s="10"/>
-      <c r="E56" s="30"/>
-      <c r="F56" s="103"/>
-      <c r="G56" s="104"/>
-      <c r="H56" s="33"/>
-      <c r="I56" s="41"/>
+      <c r="E56" s="28"/>
+      <c r="F56" s="67"/>
+      <c r="G56" s="68"/>
+      <c r="H56" s="31"/>
+      <c r="I56" s="38"/>
     </row>
     <row r="57" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="47"/>
-      <c r="B57" s="32"/>
+      <c r="A57" s="44"/>
+      <c r="B57" s="30"/>
       <c r="C57" s="11"/>
       <c r="D57" s="11"/>
       <c r="E57" s="11"/>
-      <c r="F57" s="111"/>
-      <c r="G57" s="112"/>
+      <c r="F57" s="69"/>
+      <c r="G57" s="70"/>
       <c r="H57" s="11"/>
-      <c r="I57" s="42"/>
+      <c r="I57" s="39"/>
     </row>
     <row r="58" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="47"/>
-      <c r="B58" s="33"/>
+      <c r="A58" s="44"/>
+      <c r="B58" s="31"/>
       <c r="C58" s="10"/>
-      <c r="D58" s="10"/>
-      <c r="E58" s="30"/>
-      <c r="F58" s="77"/>
-      <c r="G58" s="78"/>
-      <c r="H58" s="33"/>
-      <c r="I58" s="41"/>
+      <c r="D58" s="117"/>
+      <c r="E58" s="28"/>
+      <c r="F58" s="71"/>
+      <c r="G58" s="72"/>
+      <c r="H58" s="31"/>
+      <c r="I58" s="38"/>
     </row>
     <row r="59" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="47"/>
-      <c r="B59" s="32"/>
-      <c r="C59" s="11"/>
-      <c r="D59" s="34"/>
-      <c r="E59" s="31"/>
-      <c r="F59" s="79"/>
-      <c r="G59" s="80"/>
-      <c r="H59" s="32"/>
-      <c r="I59" s="42"/>
+      <c r="A59" s="44"/>
+      <c r="B59" s="30"/>
+      <c r="C59" s="29"/>
+      <c r="D59" s="118"/>
+      <c r="E59" s="36"/>
+      <c r="F59" s="61"/>
+      <c r="G59" s="62"/>
+      <c r="H59" s="30"/>
+      <c r="I59" s="39"/>
     </row>
     <row r="60" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="47"/>
-      <c r="B60" s="33"/>
-      <c r="C60" s="30"/>
-      <c r="D60" s="36"/>
-      <c r="E60" s="38"/>
-      <c r="F60" s="81"/>
-      <c r="G60" s="82"/>
-      <c r="H60" s="33"/>
-      <c r="I60" s="41"/>
+      <c r="A60" s="44"/>
+      <c r="B60" s="31"/>
+      <c r="C60" s="28"/>
+      <c r="D60" s="33"/>
+      <c r="E60" s="35"/>
+      <c r="F60" s="59"/>
+      <c r="G60" s="60"/>
+      <c r="H60" s="31"/>
+      <c r="I60" s="38"/>
     </row>
     <row r="61" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="47"/>
-      <c r="B61" s="32"/>
-      <c r="C61" s="31"/>
-      <c r="D61" s="37"/>
-      <c r="E61" s="39"/>
-      <c r="F61" s="79"/>
-      <c r="G61" s="80"/>
-      <c r="H61" s="32"/>
-      <c r="I61" s="42"/>
+      <c r="A61" s="44"/>
+      <c r="B61" s="30"/>
+      <c r="C61" s="29"/>
+      <c r="D61" s="34"/>
+      <c r="E61" s="36"/>
+      <c r="F61" s="61"/>
+      <c r="G61" s="62"/>
+      <c r="H61" s="30"/>
+      <c r="I61" s="39"/>
     </row>
     <row r="62" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="47"/>
-      <c r="B62" s="33"/>
-      <c r="C62" s="10"/>
-      <c r="D62" s="35"/>
-      <c r="E62" s="30"/>
-      <c r="F62" s="81"/>
-      <c r="G62" s="82"/>
-      <c r="H62" s="33"/>
-      <c r="I62" s="41"/>
+      <c r="A62" s="44"/>
+      <c r="B62" s="31"/>
+      <c r="C62" s="28"/>
+      <c r="D62" s="116"/>
+      <c r="E62" s="35"/>
+      <c r="F62" s="59"/>
+      <c r="G62" s="60"/>
+      <c r="H62" s="31"/>
+      <c r="I62" s="38"/>
     </row>
     <row r="63" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="47"/>
-      <c r="B63" s="32"/>
-      <c r="C63" s="31"/>
-      <c r="D63" s="37"/>
-      <c r="E63" s="39"/>
-      <c r="F63" s="79"/>
-      <c r="G63" s="80"/>
-      <c r="H63" s="32"/>
-      <c r="I63" s="42"/>
+      <c r="A63" s="44"/>
+      <c r="B63" s="30"/>
+      <c r="C63" s="29"/>
+      <c r="D63" s="119"/>
+      <c r="E63" s="36"/>
+      <c r="F63" s="61"/>
+      <c r="G63" s="62"/>
+      <c r="H63" s="30"/>
+      <c r="I63" s="39"/>
     </row>
     <row r="64" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="47"/>
-      <c r="B64" s="33"/>
-      <c r="C64" s="10"/>
-      <c r="D64" s="35"/>
-      <c r="E64" s="30"/>
-      <c r="F64" s="81"/>
-      <c r="G64" s="82"/>
-      <c r="H64" s="33"/>
-      <c r="I64" s="41"/>
+      <c r="A64" s="44"/>
+      <c r="B64" s="31"/>
+      <c r="C64" s="38"/>
+      <c r="D64" s="120"/>
+      <c r="E64" s="35"/>
+      <c r="F64" s="57"/>
+      <c r="G64" s="58"/>
+      <c r="H64" s="31"/>
+      <c r="I64" s="38"/>
     </row>
     <row r="65" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="47"/>
-      <c r="B65" s="32"/>
-      <c r="C65" s="31"/>
-      <c r="D65" s="37"/>
-      <c r="E65" s="39"/>
-      <c r="F65" s="79"/>
-      <c r="G65" s="80"/>
-      <c r="H65" s="32"/>
-      <c r="I65" s="42"/>
+      <c r="A65" s="44"/>
+      <c r="B65" s="30"/>
+      <c r="C65" s="39"/>
+      <c r="D65" s="119"/>
+      <c r="E65" s="36"/>
+      <c r="F65" s="61"/>
+      <c r="G65" s="62"/>
+      <c r="H65" s="30"/>
+      <c r="I65" s="39"/>
     </row>
     <row r="66" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="47"/>
-      <c r="B66" s="33"/>
-      <c r="C66" s="10"/>
-      <c r="D66" s="35"/>
-      <c r="E66" s="30"/>
-      <c r="F66" s="81"/>
-      <c r="G66" s="82"/>
-      <c r="H66" s="33"/>
-      <c r="I66" s="41"/>
+      <c r="A66" s="44"/>
+      <c r="B66" s="31"/>
+      <c r="C66" s="38"/>
+      <c r="D66" s="120"/>
+      <c r="E66" s="35"/>
+      <c r="F66" s="57"/>
+      <c r="G66" s="58"/>
+      <c r="H66" s="31"/>
+      <c r="I66" s="38"/>
     </row>
     <row r="67" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="47"/>
-      <c r="B67" s="32"/>
-      <c r="C67" s="31"/>
-      <c r="D67" s="37"/>
-      <c r="E67" s="39"/>
-      <c r="F67" s="79"/>
-      <c r="G67" s="80"/>
-      <c r="H67" s="32"/>
-      <c r="I67" s="42"/>
+      <c r="A67" s="44"/>
+      <c r="B67" s="30"/>
+      <c r="C67" s="39"/>
+      <c r="D67" s="119"/>
+      <c r="E67" s="36"/>
+      <c r="F67" s="61"/>
+      <c r="G67" s="62"/>
+      <c r="H67" s="30"/>
+      <c r="I67" s="39"/>
     </row>
     <row r="68" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="47"/>
-      <c r="B68" s="33"/>
-      <c r="C68" s="10"/>
-      <c r="D68" s="35"/>
-      <c r="E68" s="30"/>
-      <c r="F68" s="81"/>
-      <c r="G68" s="82"/>
-      <c r="H68" s="33"/>
-      <c r="I68" s="41"/>
+      <c r="A68" s="44"/>
+      <c r="B68" s="31"/>
+      <c r="C68" s="38"/>
+      <c r="D68" s="120"/>
+      <c r="E68" s="35"/>
+      <c r="F68" s="57"/>
+      <c r="G68" s="58"/>
+      <c r="H68" s="31"/>
+      <c r="I68" s="38"/>
     </row>
     <row r="69" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="47"/>
-      <c r="B69" s="32"/>
-      <c r="C69" s="31"/>
-      <c r="D69" s="37"/>
-      <c r="E69" s="39"/>
-      <c r="F69" s="79"/>
-      <c r="G69" s="80"/>
-      <c r="H69" s="32"/>
-      <c r="I69" s="42"/>
+      <c r="A69" s="44"/>
+      <c r="B69" s="30"/>
+      <c r="C69" s="39"/>
+      <c r="D69" s="119"/>
+      <c r="E69" s="36"/>
+      <c r="F69" s="61"/>
+      <c r="G69" s="62"/>
+      <c r="H69" s="30"/>
+      <c r="I69" s="39"/>
     </row>
     <row r="70" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="47"/>
-      <c r="B70" s="33"/>
-      <c r="C70" s="10"/>
-      <c r="D70" s="35"/>
-      <c r="E70" s="30"/>
-      <c r="F70" s="81"/>
-      <c r="G70" s="82"/>
-      <c r="H70" s="33"/>
-      <c r="I70" s="41"/>
-    </row>
-    <row r="71" spans="1:10" ht="22" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="47"/>
-      <c r="B71" s="62" t="s">
+      <c r="A70" s="44"/>
+      <c r="B70" s="31"/>
+      <c r="C70" s="38"/>
+      <c r="D70" s="121"/>
+      <c r="E70" s="35"/>
+      <c r="F70" s="57"/>
+      <c r="G70" s="58"/>
+      <c r="H70" s="31"/>
+      <c r="I70" s="38"/>
+    </row>
+    <row r="71" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A71" s="44"/>
+      <c r="B71" s="30"/>
+      <c r="C71" s="29"/>
+      <c r="D71" s="34"/>
+      <c r="E71" s="36"/>
+      <c r="F71" s="61"/>
+      <c r="G71" s="62"/>
+      <c r="H71" s="30"/>
+      <c r="I71" s="39"/>
+    </row>
+    <row r="72" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A72" s="44"/>
+      <c r="B72" s="31"/>
+      <c r="C72" s="10"/>
+      <c r="D72" s="32"/>
+      <c r="E72" s="28"/>
+      <c r="F72" s="59"/>
+      <c r="G72" s="60"/>
+      <c r="H72" s="31"/>
+      <c r="I72" s="38"/>
+    </row>
+    <row r="73" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A73" s="44"/>
+      <c r="B73" s="30"/>
+      <c r="C73" s="29"/>
+      <c r="D73" s="34"/>
+      <c r="E73" s="36"/>
+      <c r="F73" s="61"/>
+      <c r="G73" s="62"/>
+      <c r="H73" s="30"/>
+      <c r="I73" s="39"/>
+    </row>
+    <row r="74" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A74" s="44"/>
+      <c r="B74" s="31"/>
+      <c r="C74" s="10"/>
+      <c r="D74" s="32"/>
+      <c r="E74" s="28"/>
+      <c r="F74" s="59"/>
+      <c r="G74" s="60"/>
+      <c r="H74" s="31"/>
+      <c r="I74" s="38"/>
+    </row>
+    <row r="75" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A75" s="44"/>
+      <c r="B75" s="30"/>
+      <c r="C75" s="29"/>
+      <c r="D75" s="34"/>
+      <c r="E75" s="36"/>
+      <c r="F75" s="61"/>
+      <c r="G75" s="62"/>
+      <c r="H75" s="30"/>
+      <c r="I75" s="39"/>
+    </row>
+    <row r="76" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A76" s="44"/>
+      <c r="B76" s="31"/>
+      <c r="C76" s="10"/>
+      <c r="D76" s="32"/>
+      <c r="E76" s="28"/>
+      <c r="F76" s="59"/>
+      <c r="G76" s="60"/>
+      <c r="H76" s="31"/>
+      <c r="I76" s="38"/>
+    </row>
+    <row r="77" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A77" s="44"/>
+      <c r="B77" s="30"/>
+      <c r="C77" s="29"/>
+      <c r="D77" s="34"/>
+      <c r="E77" s="36"/>
+      <c r="F77" s="61"/>
+      <c r="G77" s="62"/>
+      <c r="H77" s="30"/>
+      <c r="I77" s="39"/>
+    </row>
+    <row r="78" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A78" s="44"/>
+      <c r="B78" s="31"/>
+      <c r="C78" s="10"/>
+      <c r="D78" s="32"/>
+      <c r="E78" s="28"/>
+      <c r="F78" s="59"/>
+      <c r="G78" s="60"/>
+      <c r="H78" s="31"/>
+      <c r="I78" s="38"/>
+    </row>
+    <row r="79" spans="1:10" ht="22" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="44"/>
+      <c r="B79" s="99" t="s">
         <v>26</v>
       </c>
-      <c r="C71" s="63"/>
-      <c r="D71" s="63"/>
-      <c r="E71" s="64"/>
-      <c r="F71" s="113">
-        <f>SUM(F9:F70)</f>
+      <c r="C79" s="100"/>
+      <c r="D79" s="100"/>
+      <c r="E79" s="101"/>
+      <c r="F79" s="63">
+        <f>SUM(F9:F78)</f>
         <v>2260</v>
       </c>
-      <c r="G71" s="114"/>
-      <c r="H71" s="50">
-        <f>SUM(H9:H70)</f>
+      <c r="G79" s="64"/>
+      <c r="H79" s="47">
+        <f>SUM(H9:H78)</f>
         <v>1031.3</v>
       </c>
-      <c r="I71" s="51">
-        <f>SUM(I9:I70)</f>
+      <c r="I79" s="48">
+        <f>SUM(I9:I78)</f>
         <v>3291.3</v>
       </c>
-      <c r="J71" s="49"/>
-    </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B73" s="60" t="s">
+      <c r="J79" s="46"/>
+    </row>
+    <row r="81" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B81" s="97" t="s">
         <v>27</v>
       </c>
-      <c r="C73" s="61"/>
-      <c r="D73" s="61"/>
-      <c r="E73" s="61"/>
-      <c r="F73" s="61"/>
-      <c r="G73" s="61"/>
-      <c r="H73" s="61"/>
-      <c r="I73" s="61"/>
+      <c r="C81" s="98"/>
+      <c r="D81" s="98"/>
+      <c r="E81" s="98"/>
+      <c r="F81" s="98"/>
+      <c r="G81" s="98"/>
+      <c r="H81" s="98"/>
+      <c r="I81" s="98"/>
     </row>
   </sheetData>
-  <mergeCells count="74">
-    <mergeCell ref="F60:G60"/>
-    <mergeCell ref="F61:G61"/>
-    <mergeCell ref="F62:G62"/>
-    <mergeCell ref="F70:G70"/>
-    <mergeCell ref="F71:G71"/>
-    <mergeCell ref="F63:G63"/>
-    <mergeCell ref="F64:G64"/>
-    <mergeCell ref="F66:G66"/>
-    <mergeCell ref="F67:G67"/>
-    <mergeCell ref="F69:G69"/>
-    <mergeCell ref="F65:G65"/>
-    <mergeCell ref="F68:G68"/>
-    <mergeCell ref="F49:G49"/>
-    <mergeCell ref="F50:G50"/>
-    <mergeCell ref="F51:G51"/>
-    <mergeCell ref="F58:G58"/>
-    <mergeCell ref="F59:G59"/>
-    <mergeCell ref="F52:G52"/>
-    <mergeCell ref="F53:G53"/>
-    <mergeCell ref="F54:G54"/>
-    <mergeCell ref="F55:G55"/>
-    <mergeCell ref="F56:G56"/>
-    <mergeCell ref="F57:G57"/>
-    <mergeCell ref="F44:G44"/>
-    <mergeCell ref="F45:G45"/>
-    <mergeCell ref="F46:G46"/>
-    <mergeCell ref="F47:G47"/>
-    <mergeCell ref="F48:G48"/>
-    <mergeCell ref="F39:G39"/>
-    <mergeCell ref="F40:G40"/>
-    <mergeCell ref="F41:G41"/>
-    <mergeCell ref="F42:G42"/>
-    <mergeCell ref="F43:G43"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="F35:G35"/>
-    <mergeCell ref="F36:G36"/>
-    <mergeCell ref="F37:G37"/>
-    <mergeCell ref="F38:G38"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="F23:G23"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B3:I3"/>
-    <mergeCell ref="E4:G4"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="B73:I73"/>
-    <mergeCell ref="B71:E71"/>
+  <mergeCells count="78">
+    <mergeCell ref="B81:I81"/>
+    <mergeCell ref="B79:E79"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="H4:I4"/>
@@ -2401,6 +2473,68 @@
     <mergeCell ref="F16:G16"/>
     <mergeCell ref="F17:G17"/>
     <mergeCell ref="F18:G18"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="E4:G4"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="F23:G23"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="F38:G38"/>
+    <mergeCell ref="F39:G39"/>
+    <mergeCell ref="F40:G40"/>
+    <mergeCell ref="F41:G41"/>
+    <mergeCell ref="F42:G42"/>
+    <mergeCell ref="F43:G43"/>
+    <mergeCell ref="F44:G44"/>
+    <mergeCell ref="F45:G45"/>
+    <mergeCell ref="F46:G46"/>
+    <mergeCell ref="F47:G47"/>
+    <mergeCell ref="F48:G48"/>
+    <mergeCell ref="F49:G49"/>
+    <mergeCell ref="F50:G50"/>
+    <mergeCell ref="F51:G51"/>
+    <mergeCell ref="F58:G58"/>
+    <mergeCell ref="F59:G59"/>
+    <mergeCell ref="F52:G52"/>
+    <mergeCell ref="F53:G53"/>
+    <mergeCell ref="F54:G54"/>
+    <mergeCell ref="F55:G55"/>
+    <mergeCell ref="F56:G56"/>
+    <mergeCell ref="F57:G57"/>
+    <mergeCell ref="F60:G60"/>
+    <mergeCell ref="F61:G61"/>
+    <mergeCell ref="F62:G62"/>
+    <mergeCell ref="F78:G78"/>
+    <mergeCell ref="F79:G79"/>
+    <mergeCell ref="F71:G71"/>
+    <mergeCell ref="F72:G72"/>
+    <mergeCell ref="F74:G74"/>
+    <mergeCell ref="F75:G75"/>
+    <mergeCell ref="F77:G77"/>
+    <mergeCell ref="F73:G73"/>
+    <mergeCell ref="F76:G76"/>
+    <mergeCell ref="F63:G63"/>
+    <mergeCell ref="F65:G65"/>
+    <mergeCell ref="F67:G67"/>
+    <mergeCell ref="F69:G69"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2409,7 +2543,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A2:I60"/>
+  <dimension ref="A2:I75"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -2423,15 +2557,15 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:9" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="116" t="s">
+      <c r="B2" s="115" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="61"/>
-      <c r="D2" s="61"/>
-      <c r="E2" s="61"/>
-      <c r="F2" s="61"/>
-      <c r="G2" s="61"/>
-      <c r="H2" s="61"/>
+      <c r="C2" s="98"/>
+      <c r="D2" s="98"/>
+      <c r="E2" s="98"/>
+      <c r="F2" s="98"/>
+      <c r="G2" s="98"/>
+      <c r="H2" s="98"/>
     </row>
     <row r="4" spans="1:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="13"/>
@@ -2459,7 +2593,7 @@
       <c r="I4" s="13"/>
     </row>
     <row r="6" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="53" t="s">
+      <c r="B6" s="50" t="s">
         <v>12</v>
       </c>
       <c r="C6" s="1" t="s">
@@ -2468,22 +2602,22 @@
       <c r="D6" s="1">
         <v>218</v>
       </c>
-      <c r="E6" s="54" t="s">
+      <c r="E6" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="58">
+      <c r="F6" s="55">
         <v>30</v>
       </c>
-      <c r="G6" s="55">
+      <c r="G6" s="52">
         <v>32.700000000000003</v>
       </c>
-      <c r="H6" s="59">
+      <c r="H6" s="56">
         <f>F6+G6</f>
         <v>62.7</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="53" t="s">
+      <c r="B7" s="50" t="s">
         <v>15</v>
       </c>
       <c r="C7" s="1" t="s">
@@ -2492,22 +2626,22 @@
       <c r="D7" s="9">
         <v>45</v>
       </c>
-      <c r="E7" s="54" t="s">
+      <c r="E7" s="51" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="58">
+      <c r="F7" s="55">
         <v>180</v>
       </c>
-      <c r="G7" s="55">
+      <c r="G7" s="52">
         <v>40.5</v>
       </c>
-      <c r="H7" s="59">
+      <c r="H7" s="56">
         <f>F7+G7</f>
         <v>220.5</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="53" t="s">
+      <c r="B8" s="50" t="s">
         <v>17</v>
       </c>
       <c r="C8" s="1" t="s">
@@ -2516,22 +2650,22 @@
       <c r="D8" s="2">
         <v>88</v>
       </c>
-      <c r="E8" s="54" t="s">
+      <c r="E8" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="F8" s="58">
+      <c r="F8" s="55">
         <v>500</v>
       </c>
-      <c r="G8" s="55">
+      <c r="G8" s="52">
         <v>220</v>
       </c>
-      <c r="H8" s="59">
+      <c r="H8" s="56">
         <f>F8+G8</f>
         <v>720</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="53" t="s">
+      <c r="B9" s="50" t="s">
         <v>20</v>
       </c>
       <c r="C9" s="1" t="s">
@@ -2540,499 +2674,619 @@
       <c r="D9" s="2">
         <v>113</v>
       </c>
-      <c r="E9" s="54" t="s">
+      <c r="E9" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="F9" s="58">
+      <c r="F9" s="55">
         <v>1200</v>
       </c>
-      <c r="G9" s="55">
+      <c r="G9" s="52">
         <v>678.6</v>
       </c>
-      <c r="H9" s="59">
+      <c r="H9" s="56">
         <f>F9+G9</f>
         <v>1878.6</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="16"/>
-      <c r="C10" s="52"/>
-      <c r="D10" s="52"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="49"/>
+      <c r="D10" s="49"/>
       <c r="E10" s="8"/>
       <c r="F10" s="5"/>
       <c r="G10" s="6"/>
       <c r="H10" s="7"/>
     </row>
     <row r="11" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="16"/>
-      <c r="C11" s="52"/>
-      <c r="D11" s="52"/>
+      <c r="B11" s="14"/>
+      <c r="C11" s="49"/>
+      <c r="D11" s="49"/>
       <c r="E11" s="8"/>
       <c r="F11" s="5"/>
       <c r="G11" s="6"/>
       <c r="H11" s="7"/>
     </row>
     <row r="12" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="16"/>
-      <c r="C12" s="52"/>
-      <c r="D12" s="52"/>
+      <c r="B12" s="14"/>
+      <c r="C12" s="49"/>
+      <c r="D12" s="49"/>
       <c r="E12" s="8"/>
       <c r="F12" s="5"/>
       <c r="G12" s="6"/>
       <c r="H12" s="7"/>
     </row>
     <row r="13" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="16"/>
-      <c r="C13" s="52"/>
-      <c r="D13" s="52"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="49"/>
+      <c r="D13" s="49"/>
       <c r="E13" s="8"/>
       <c r="F13" s="5"/>
       <c r="G13" s="6"/>
       <c r="H13" s="7"/>
     </row>
     <row r="14" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="16"/>
-      <c r="C14" s="52"/>
-      <c r="D14" s="52"/>
+      <c r="B14" s="14"/>
+      <c r="C14" s="49"/>
+      <c r="D14" s="49"/>
       <c r="E14" s="8"/>
       <c r="F14" s="5"/>
       <c r="G14" s="6"/>
       <c r="H14" s="7"/>
     </row>
     <row r="15" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="16"/>
-      <c r="C15" s="52"/>
-      <c r="D15" s="52"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="49"/>
+      <c r="D15" s="49"/>
       <c r="E15" s="8"/>
       <c r="F15" s="5"/>
       <c r="G15" s="6"/>
       <c r="H15" s="7"/>
     </row>
     <row r="16" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="16"/>
-      <c r="C16" s="52"/>
-      <c r="D16" s="52"/>
+      <c r="B16" s="14"/>
+      <c r="C16" s="49"/>
+      <c r="D16" s="49"/>
       <c r="E16" s="8"/>
       <c r="F16" s="5"/>
       <c r="G16" s="6"/>
       <c r="H16" s="7"/>
     </row>
     <row r="17" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="16"/>
-      <c r="C17" s="52"/>
-      <c r="D17" s="52"/>
+      <c r="B17" s="14"/>
+      <c r="C17" s="49"/>
+      <c r="D17" s="49"/>
       <c r="E17" s="8"/>
       <c r="F17" s="5"/>
       <c r="G17" s="6"/>
       <c r="H17" s="7"/>
     </row>
     <row r="18" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="16"/>
-      <c r="C18" s="52"/>
-      <c r="D18" s="52"/>
+      <c r="B18" s="14"/>
+      <c r="C18" s="49"/>
+      <c r="D18" s="49"/>
       <c r="E18" s="8"/>
       <c r="F18" s="5"/>
       <c r="G18" s="6"/>
       <c r="H18" s="7"/>
     </row>
     <row r="19" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="16"/>
-      <c r="C19" s="52"/>
-      <c r="D19" s="52"/>
+      <c r="B19" s="14"/>
+      <c r="C19" s="49"/>
+      <c r="D19" s="49"/>
       <c r="E19" s="8"/>
       <c r="F19" s="5"/>
       <c r="G19" s="6"/>
       <c r="H19" s="7"/>
     </row>
     <row r="20" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="16"/>
-      <c r="C20" s="52"/>
-      <c r="D20" s="52"/>
+      <c r="B20" s="14"/>
+      <c r="C20" s="49"/>
+      <c r="D20" s="49"/>
       <c r="E20" s="8"/>
       <c r="F20" s="5"/>
       <c r="G20" s="6"/>
       <c r="H20" s="7"/>
     </row>
     <row r="21" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="16"/>
-      <c r="C21" s="52"/>
-      <c r="D21" s="52"/>
+      <c r="B21" s="14"/>
+      <c r="C21" s="49"/>
+      <c r="D21" s="49"/>
       <c r="E21" s="8"/>
       <c r="F21" s="5"/>
       <c r="G21" s="6"/>
       <c r="H21" s="7"/>
     </row>
     <row r="22" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="16"/>
-      <c r="C22" s="52"/>
-      <c r="D22" s="52"/>
+      <c r="B22" s="14"/>
+      <c r="C22" s="49"/>
+      <c r="D22" s="49"/>
       <c r="E22" s="8"/>
       <c r="F22" s="5"/>
       <c r="G22" s="6"/>
       <c r="H22" s="7"/>
     </row>
     <row r="23" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="16"/>
-      <c r="C23" s="52"/>
-      <c r="D23" s="52"/>
+      <c r="B23" s="14"/>
+      <c r="C23" s="49"/>
+      <c r="D23" s="49"/>
       <c r="E23" s="8"/>
       <c r="F23" s="5"/>
       <c r="G23" s="6"/>
       <c r="H23" s="7"/>
     </row>
     <row r="24" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="16"/>
-      <c r="C24" s="52"/>
-      <c r="D24" s="52"/>
+      <c r="B24" s="14"/>
+      <c r="C24" s="49"/>
+      <c r="D24" s="49"/>
       <c r="E24" s="8"/>
       <c r="F24" s="5"/>
       <c r="G24" s="6"/>
       <c r="H24" s="7"/>
     </row>
     <row r="25" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="16"/>
-      <c r="C25" s="52"/>
-      <c r="D25" s="52"/>
+      <c r="B25" s="14"/>
+      <c r="C25" s="49"/>
+      <c r="D25" s="49"/>
       <c r="E25" s="8"/>
       <c r="F25" s="5"/>
       <c r="G25" s="6"/>
       <c r="H25" s="7"/>
     </row>
     <row r="26" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="16"/>
-      <c r="C26" s="52"/>
-      <c r="D26" s="52"/>
+      <c r="B26" s="14"/>
+      <c r="C26" s="49"/>
+      <c r="D26" s="49"/>
       <c r="E26" s="8"/>
       <c r="F26" s="5"/>
       <c r="G26" s="6"/>
       <c r="H26" s="7"/>
     </row>
     <row r="27" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="16"/>
-      <c r="C27" s="52"/>
-      <c r="D27" s="52"/>
+      <c r="B27" s="14"/>
+      <c r="C27" s="49"/>
+      <c r="D27" s="49"/>
       <c r="E27" s="8"/>
       <c r="F27" s="5"/>
       <c r="G27" s="6"/>
       <c r="H27" s="7"/>
     </row>
     <row r="28" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B28" s="16"/>
-      <c r="C28" s="52"/>
-      <c r="D28" s="52"/>
+      <c r="B28" s="14"/>
+      <c r="C28" s="49"/>
+      <c r="D28" s="49"/>
       <c r="E28" s="8"/>
       <c r="F28" s="5"/>
       <c r="G28" s="6"/>
       <c r="H28" s="7"/>
     </row>
     <row r="29" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B29" s="16"/>
-      <c r="C29" s="52"/>
-      <c r="D29" s="52"/>
+      <c r="B29" s="14"/>
+      <c r="C29" s="49"/>
+      <c r="D29" s="49"/>
       <c r="E29" s="8"/>
       <c r="F29" s="5"/>
       <c r="G29" s="6"/>
       <c r="H29" s="7"/>
     </row>
     <row r="30" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B30" s="16"/>
-      <c r="C30" s="52"/>
-      <c r="D30" s="52"/>
+      <c r="B30" s="14"/>
+      <c r="C30" s="49"/>
+      <c r="D30" s="49"/>
       <c r="E30" s="8"/>
       <c r="F30" s="5"/>
       <c r="G30" s="6"/>
       <c r="H30" s="7"/>
     </row>
     <row r="31" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="16"/>
-      <c r="C31" s="52"/>
-      <c r="D31" s="52"/>
+      <c r="B31" s="14"/>
+      <c r="C31" s="49"/>
+      <c r="D31" s="49"/>
       <c r="E31" s="8"/>
       <c r="F31" s="5"/>
       <c r="G31" s="6"/>
       <c r="H31" s="7"/>
     </row>
     <row r="32" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="16"/>
-      <c r="C32" s="52"/>
-      <c r="D32" s="52"/>
+      <c r="B32" s="14"/>
+      <c r="C32" s="49"/>
+      <c r="D32" s="49"/>
       <c r="E32" s="8"/>
       <c r="F32" s="5"/>
       <c r="G32" s="6"/>
       <c r="H32" s="7"/>
     </row>
     <row r="33" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B33" s="16"/>
-      <c r="C33" s="52"/>
-      <c r="D33" s="52"/>
+      <c r="B33" s="14"/>
+      <c r="C33" s="49"/>
+      <c r="D33" s="49"/>
       <c r="E33" s="8"/>
       <c r="F33" s="5"/>
       <c r="G33" s="6"/>
       <c r="H33" s="7"/>
     </row>
     <row r="34" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B34" s="16"/>
-      <c r="C34" s="52"/>
-      <c r="D34" s="52"/>
+      <c r="B34" s="14"/>
+      <c r="C34" s="49"/>
+      <c r="D34" s="49"/>
       <c r="E34" s="8"/>
       <c r="F34" s="5"/>
       <c r="G34" s="6"/>
       <c r="H34" s="7"/>
     </row>
     <row r="35" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="16"/>
-      <c r="C35" s="52"/>
-      <c r="D35" s="52"/>
+      <c r="B35" s="14"/>
+      <c r="C35" s="49"/>
+      <c r="D35" s="49"/>
       <c r="E35" s="8"/>
       <c r="F35" s="5"/>
       <c r="G35" s="6"/>
       <c r="H35" s="7"/>
     </row>
     <row r="36" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B36" s="16"/>
-      <c r="C36" s="52"/>
-      <c r="D36" s="52"/>
+      <c r="B36" s="14"/>
+      <c r="C36" s="49"/>
+      <c r="D36" s="49"/>
       <c r="E36" s="8"/>
       <c r="F36" s="5"/>
       <c r="G36" s="6"/>
       <c r="H36" s="7"/>
     </row>
     <row r="37" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B37" s="16"/>
-      <c r="C37" s="52"/>
-      <c r="D37" s="52"/>
+      <c r="B37" s="14"/>
+      <c r="C37" s="49"/>
+      <c r="D37" s="49"/>
       <c r="E37" s="8"/>
       <c r="F37" s="5"/>
       <c r="G37" s="6"/>
       <c r="H37" s="7"/>
     </row>
     <row r="38" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B38" s="16"/>
-      <c r="C38" s="52"/>
-      <c r="D38" s="52"/>
+      <c r="B38" s="14"/>
+      <c r="C38" s="49"/>
+      <c r="D38" s="49"/>
       <c r="E38" s="8"/>
       <c r="F38" s="5"/>
       <c r="G38" s="6"/>
       <c r="H38" s="7"/>
     </row>
     <row r="39" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B39" s="16"/>
-      <c r="C39" s="52"/>
-      <c r="D39" s="52"/>
+      <c r="B39" s="14"/>
+      <c r="C39" s="49"/>
+      <c r="D39" s="49"/>
       <c r="E39" s="8"/>
       <c r="F39" s="5"/>
       <c r="G39" s="6"/>
       <c r="H39" s="7"/>
     </row>
     <row r="40" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B40" s="16"/>
-      <c r="C40" s="52"/>
-      <c r="D40" s="52"/>
+      <c r="B40" s="14"/>
+      <c r="C40" s="49"/>
+      <c r="D40" s="49"/>
       <c r="E40" s="8"/>
       <c r="F40" s="5"/>
       <c r="G40" s="6"/>
       <c r="H40" s="7"/>
     </row>
     <row r="41" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B41" s="16"/>
-      <c r="C41" s="52"/>
-      <c r="D41" s="52"/>
+      <c r="B41" s="14"/>
+      <c r="C41" s="49"/>
+      <c r="D41" s="49"/>
       <c r="E41" s="8"/>
       <c r="F41" s="5"/>
       <c r="G41" s="6"/>
       <c r="H41" s="7"/>
     </row>
     <row r="42" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B42" s="16"/>
-      <c r="C42" s="52"/>
-      <c r="D42" s="52"/>
+      <c r="B42" s="14"/>
+      <c r="C42" s="49"/>
+      <c r="D42" s="49"/>
       <c r="E42" s="8"/>
       <c r="F42" s="5"/>
       <c r="G42" s="6"/>
       <c r="H42" s="7"/>
     </row>
     <row r="43" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B43" s="16"/>
-      <c r="C43" s="52"/>
-      <c r="D43" s="52"/>
+      <c r="B43" s="14"/>
+      <c r="C43" s="49"/>
+      <c r="D43" s="49"/>
       <c r="E43" s="8"/>
       <c r="F43" s="5"/>
       <c r="G43" s="6"/>
       <c r="H43" s="7"/>
     </row>
     <row r="44" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B44" s="16"/>
-      <c r="C44" s="52"/>
-      <c r="D44" s="52"/>
+      <c r="B44" s="14"/>
+      <c r="C44" s="49"/>
+      <c r="D44" s="49"/>
       <c r="E44" s="8"/>
       <c r="F44" s="5"/>
       <c r="G44" s="6"/>
       <c r="H44" s="7"/>
     </row>
     <row r="45" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B45" s="16"/>
-      <c r="C45" s="52"/>
-      <c r="D45" s="52"/>
+      <c r="B45" s="14"/>
+      <c r="C45" s="49"/>
+      <c r="D45" s="49"/>
       <c r="E45" s="8"/>
       <c r="F45" s="5"/>
       <c r="G45" s="6"/>
       <c r="H45" s="7"/>
     </row>
     <row r="46" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B46" s="16"/>
-      <c r="C46" s="52"/>
-      <c r="D46" s="52"/>
+      <c r="B46" s="14"/>
+      <c r="C46" s="49"/>
+      <c r="D46" s="49"/>
       <c r="E46" s="8"/>
       <c r="F46" s="5"/>
       <c r="G46" s="6"/>
       <c r="H46" s="7"/>
     </row>
     <row r="47" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B47" s="16"/>
-      <c r="C47" s="52"/>
-      <c r="D47" s="52"/>
+      <c r="B47" s="14"/>
+      <c r="C47" s="49"/>
+      <c r="D47" s="49"/>
       <c r="E47" s="8"/>
       <c r="F47" s="5"/>
       <c r="G47" s="6"/>
       <c r="H47" s="7"/>
     </row>
     <row r="48" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B48" s="16"/>
-      <c r="C48" s="52"/>
-      <c r="D48" s="52"/>
+      <c r="B48" s="14"/>
+      <c r="C48" s="49"/>
+      <c r="D48" s="49"/>
       <c r="E48" s="8"/>
       <c r="F48" s="5"/>
       <c r="G48" s="6"/>
       <c r="H48" s="7"/>
     </row>
     <row r="49" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B49" s="16"/>
-      <c r="C49" s="52"/>
-      <c r="D49" s="52"/>
+      <c r="B49" s="14"/>
+      <c r="C49" s="49"/>
+      <c r="D49" s="49"/>
       <c r="E49" s="8"/>
       <c r="F49" s="5"/>
       <c r="G49" s="6"/>
       <c r="H49" s="7"/>
     </row>
     <row r="50" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B50" s="16"/>
-      <c r="C50" s="52"/>
-      <c r="D50" s="52"/>
+      <c r="B50" s="14"/>
+      <c r="C50" s="49"/>
+      <c r="D50" s="49"/>
       <c r="E50" s="8"/>
       <c r="F50" s="5"/>
       <c r="G50" s="6"/>
       <c r="H50" s="7"/>
     </row>
     <row r="51" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B51" s="16"/>
-      <c r="C51" s="52"/>
-      <c r="D51" s="52"/>
+      <c r="B51" s="14"/>
+      <c r="C51" s="49"/>
+      <c r="D51" s="49"/>
       <c r="E51" s="8"/>
       <c r="F51" s="5"/>
       <c r="G51" s="6"/>
       <c r="H51" s="7"/>
     </row>
     <row r="52" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B52" s="16"/>
-      <c r="C52" s="52"/>
-      <c r="D52" s="52"/>
+      <c r="B52" s="14"/>
+      <c r="C52" s="49"/>
+      <c r="D52" s="49"/>
       <c r="E52" s="8"/>
       <c r="F52" s="5"/>
       <c r="G52" s="6"/>
       <c r="H52" s="7"/>
     </row>
     <row r="53" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B53" s="16"/>
-      <c r="C53" s="52"/>
-      <c r="D53" s="52"/>
+      <c r="B53" s="14"/>
+      <c r="C53" s="49"/>
+      <c r="D53" s="49"/>
       <c r="E53" s="8"/>
       <c r="F53" s="5"/>
       <c r="G53" s="6"/>
       <c r="H53" s="7"/>
     </row>
     <row r="54" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B54" s="16"/>
-      <c r="C54" s="52"/>
-      <c r="D54" s="52"/>
+      <c r="B54" s="14"/>
+      <c r="C54" s="49"/>
+      <c r="D54" s="49"/>
       <c r="E54" s="8"/>
       <c r="F54" s="5"/>
       <c r="G54" s="6"/>
       <c r="H54" s="7"/>
     </row>
     <row r="55" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B55" s="16"/>
-      <c r="C55" s="52"/>
-      <c r="D55" s="52"/>
+      <c r="B55" s="14"/>
+      <c r="C55" s="49"/>
+      <c r="D55" s="49"/>
       <c r="E55" s="8"/>
       <c r="F55" s="5"/>
       <c r="G55" s="6"/>
       <c r="H55" s="7"/>
     </row>
     <row r="56" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B56" s="16"/>
-      <c r="C56" s="52"/>
-      <c r="D56" s="52"/>
+      <c r="B56" s="14"/>
+      <c r="C56" s="49"/>
+      <c r="D56" s="49"/>
       <c r="E56" s="8"/>
       <c r="F56" s="5"/>
       <c r="G56" s="6"/>
       <c r="H56" s="7"/>
     </row>
     <row r="57" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B57" s="16"/>
-      <c r="C57" s="52"/>
-      <c r="D57" s="52"/>
+      <c r="B57" s="14"/>
+      <c r="C57" s="49"/>
+      <c r="D57" s="49"/>
       <c r="E57" s="8"/>
       <c r="F57" s="5"/>
       <c r="G57" s="6"/>
       <c r="H57" s="7"/>
     </row>
     <row r="58" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B58" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="C58" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D58" s="9">
-        <v>34</v>
-      </c>
-      <c r="E58" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="F58" s="5">
-        <v>350</v>
-      </c>
-      <c r="G58" s="6">
-        <v>59.5</v>
-      </c>
-      <c r="H58" s="7">
-        <f>F58+G58</f>
-        <v>409.5</v>
-      </c>
-    </row>
-    <row r="60" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B60" s="115" t="s">
+      <c r="B58" s="14"/>
+      <c r="C58" s="49"/>
+      <c r="D58" s="49"/>
+      <c r="E58" s="8"/>
+      <c r="F58" s="5"/>
+      <c r="G58" s="6"/>
+      <c r="H58" s="7"/>
+    </row>
+    <row r="59" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B59" s="14"/>
+      <c r="C59" s="49"/>
+      <c r="D59" s="49"/>
+      <c r="E59" s="8"/>
+      <c r="F59" s="5"/>
+      <c r="G59" s="6"/>
+      <c r="H59" s="7"/>
+    </row>
+    <row r="60" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B60" s="14"/>
+      <c r="C60" s="49"/>
+      <c r="D60" s="49"/>
+      <c r="E60" s="8"/>
+      <c r="F60" s="5"/>
+      <c r="G60" s="6"/>
+      <c r="H60" s="7"/>
+    </row>
+    <row r="61" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B61" s="14"/>
+      <c r="C61" s="49"/>
+      <c r="D61" s="49"/>
+      <c r="E61" s="8"/>
+      <c r="F61" s="5"/>
+      <c r="G61" s="6"/>
+      <c r="H61" s="7"/>
+    </row>
+    <row r="62" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B62" s="14"/>
+      <c r="C62" s="49"/>
+      <c r="D62" s="49"/>
+      <c r="E62" s="8"/>
+      <c r="F62" s="5"/>
+      <c r="G62" s="6"/>
+      <c r="H62" s="7"/>
+    </row>
+    <row r="63" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B63" s="14"/>
+      <c r="C63" s="49"/>
+      <c r="D63" s="49"/>
+      <c r="E63" s="8"/>
+      <c r="F63" s="5"/>
+      <c r="G63" s="6"/>
+      <c r="H63" s="7"/>
+    </row>
+    <row r="64" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B64" s="14"/>
+      <c r="C64" s="49"/>
+      <c r="D64" s="49"/>
+      <c r="E64" s="8"/>
+      <c r="F64" s="5"/>
+      <c r="G64" s="6"/>
+      <c r="H64" s="7"/>
+    </row>
+    <row r="65" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B65" s="14"/>
+      <c r="C65" s="49"/>
+      <c r="D65" s="49"/>
+      <c r="E65" s="8"/>
+      <c r="F65" s="5"/>
+      <c r="G65" s="6"/>
+      <c r="H65" s="7"/>
+    </row>
+    <row r="66" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B66" s="14"/>
+      <c r="C66" s="49"/>
+      <c r="D66" s="49"/>
+      <c r="E66" s="8"/>
+      <c r="F66" s="5"/>
+      <c r="G66" s="6"/>
+      <c r="H66" s="7"/>
+    </row>
+    <row r="67" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B67" s="14"/>
+      <c r="C67" s="49"/>
+      <c r="D67" s="49"/>
+      <c r="E67" s="8"/>
+      <c r="F67" s="5"/>
+      <c r="G67" s="6"/>
+      <c r="H67" s="7"/>
+    </row>
+    <row r="68" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B68" s="14"/>
+      <c r="C68" s="49"/>
+      <c r="D68" s="49"/>
+      <c r="E68" s="8"/>
+      <c r="F68" s="5"/>
+      <c r="G68" s="6"/>
+      <c r="H68" s="7"/>
+    </row>
+    <row r="69" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B69" s="14"/>
+      <c r="C69" s="49"/>
+      <c r="D69" s="49"/>
+      <c r="E69" s="8"/>
+      <c r="F69" s="5"/>
+      <c r="G69" s="6"/>
+      <c r="H69" s="7"/>
+    </row>
+    <row r="70" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B70" s="14"/>
+      <c r="C70" s="49"/>
+      <c r="D70" s="49"/>
+      <c r="E70" s="8"/>
+      <c r="F70" s="5"/>
+      <c r="G70" s="6"/>
+      <c r="H70" s="7"/>
+    </row>
+    <row r="71" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B71" s="14"/>
+      <c r="C71" s="49"/>
+      <c r="D71" s="49"/>
+      <c r="E71" s="8"/>
+      <c r="F71" s="5"/>
+      <c r="G71" s="6"/>
+      <c r="H71" s="7"/>
+    </row>
+    <row r="72" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B72" s="14"/>
+      <c r="C72" s="49"/>
+      <c r="D72" s="49"/>
+      <c r="E72" s="8"/>
+      <c r="F72" s="5"/>
+      <c r="G72" s="6"/>
+      <c r="H72" s="7"/>
+    </row>
+    <row r="73" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B73" s="14"/>
+      <c r="C73" s="49"/>
+      <c r="D73" s="49"/>
+      <c r="E73" s="8"/>
+      <c r="F73" s="5"/>
+      <c r="G73" s="6"/>
+      <c r="H73" s="7"/>
+    </row>
+    <row r="75" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B75" s="114" t="s">
         <v>31</v>
       </c>
-      <c r="C60" s="61"/>
-      <c r="D60" s="61"/>
-      <c r="E60" s="61"/>
-      <c r="F60" s="12">
-        <f>SUM(F6:F59)</f>
-        <v>2260</v>
-      </c>
-      <c r="G60" s="12">
-        <f>SUM(G6:G59)</f>
-        <v>1031.3</v>
-      </c>
-      <c r="H60" s="12">
-        <f>SUM(H6:H59)</f>
-        <v>3291.3</v>
+      <c r="C75" s="98"/>
+      <c r="D75" s="98"/>
+      <c r="E75" s="98"/>
+      <c r="F75" s="12">
+        <f>SUM(F6:F74)</f>
+        <v>1910</v>
+      </c>
+      <c r="G75" s="12">
+        <f>SUM(G6:G74)</f>
+        <v>971.8</v>
+      </c>
+      <c r="H75" s="12">
+        <f>SUM(H6:H74)</f>
+        <v>2881.8</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B60:E60"/>
+    <mergeCell ref="B75:E75"/>
     <mergeCell ref="B2:H2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3052,13 +3306,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="116" t="s">
+      <c r="B2" s="115" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="61"/>
-      <c r="D2" s="61"/>
-      <c r="E2" s="61"/>
-      <c r="F2" s="61"/>
+      <c r="C2" s="98"/>
+      <c r="D2" s="98"/>
+      <c r="E2" s="98"/>
+      <c r="F2" s="98"/>
     </row>
     <row r="4" spans="1:7" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="13"/>
@@ -3080,10 +3334,10 @@
       <c r="G4" s="13"/>
     </row>
     <row r="6" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="C6" s="18">
+      <c r="C6" s="16">
         <v>0</v>
       </c>
       <c r="D6" s="5">
@@ -3098,10 +3352,10 @@
       </c>
     </row>
     <row r="7" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="C7" s="18">
+      <c r="C7" s="16">
         <v>0</v>
       </c>
       <c r="D7" s="5">
@@ -3116,10 +3370,10 @@
       </c>
     </row>
     <row r="8" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="18">
+      <c r="C8" s="16">
         <v>0</v>
       </c>
       <c r="D8" s="5">
@@ -3134,10 +3388,10 @@
       </c>
     </row>
     <row r="9" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="C9" s="18">
+      <c r="C9" s="16">
         <v>0</v>
       </c>
       <c r="D9" s="5">
@@ -3152,10 +3406,10 @@
       </c>
     </row>
     <row r="10" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="22" t="s">
+      <c r="B10" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="C10" s="18">
+      <c r="C10" s="16">
         <v>0</v>
       </c>
       <c r="D10" s="5">
@@ -3170,10 +3424,10 @@
       </c>
     </row>
     <row r="11" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="23" t="s">
+      <c r="B11" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="C11" s="18">
+      <c r="C11" s="16">
         <v>1</v>
       </c>
       <c r="D11" s="5">
@@ -3188,10 +3442,10 @@
       </c>
     </row>
     <row r="12" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="24" t="s">
+      <c r="B12" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="18">
+      <c r="C12" s="16">
         <v>1</v>
       </c>
       <c r="D12" s="5">
@@ -3206,10 +3460,10 @@
       </c>
     </row>
     <row r="13" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="25" t="s">
+      <c r="B13" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="18">
+      <c r="C13" s="16">
         <v>1</v>
       </c>
       <c r="D13" s="5">
@@ -3224,10 +3478,10 @@
       </c>
     </row>
     <row r="14" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="26" t="s">
+      <c r="B14" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="18">
+      <c r="C14" s="16">
         <v>3</v>
       </c>
       <c r="D14" s="5">
@@ -3242,10 +3496,10 @@
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B16" s="115" t="s">
+      <c r="B16" s="114" t="s">
         <v>39</v>
       </c>
-      <c r="C16" s="61"/>
+      <c r="C16" s="98"/>
       <c r="D16" s="12">
         <f>SUM(D6:D15)</f>
         <v>2260</v>

</xml_diff>